<commit_message>
refactor: implement dynamic algorithm factory and modular RMSCA subpackages
- Organized com.snets2.rmsca into routing, modulation, spectrum, and core subpackages.
- Enhanced AlgorithmFactory to support registry-based instantiation for all RCSA sub-algorithms.
- Standardized IModulationSelection to be stateless, fetching parameters from ControlPlane.
- Refactored StandardIntegratedRMSCA to use dynamic injection of sub-algorithms.
- Renamed 'integratedRmlsa' to 'integratedRMSCA' for terminological consistency.
- Updated ExperimentalPlanner and unit tests to align with the new architecture.
</commit_message>
<xml_diff>
--- a/experiments/experiment01/results.xlsx
+++ b/experiments/experiment01/results.xlsx
@@ -830,13 +830,13 @@
         <v>16</v>
       </c>
       <c r="F26" t="n" s="0">
-        <v>2.5333692227306554E-4</v>
+        <v>3.80041487862425E-4</v>
       </c>
       <c r="G26" t="n" s="0">
-        <v>2.5534631343759976E-4</v>
+        <v>1.276466740063504E-4</v>
       </c>
       <c r="H26" t="n" s="0">
-        <v>0.0</v>
+        <v>5.119754251795914E-4</v>
       </c>
     </row>
     <row r="27">
@@ -856,13 +856,13 @@
         <v>17</v>
       </c>
       <c r="F27" t="n" s="0">
-        <v>1.2785884383640462E-4</v>
+        <v>2.555828887255998E-4</v>
       </c>
       <c r="G27" t="n" s="0">
-        <v>0.0</v>
+        <v>1.295231927467012E-4</v>
       </c>
       <c r="H27" t="n" s="0">
-        <v>1.2971640750409418E-4</v>
+        <v>2.597782143494991E-4</v>
       </c>
     </row>
     <row r="28">
@@ -882,13 +882,13 @@
         <v>15</v>
       </c>
       <c r="F28" t="n" s="0">
-        <v>3.876094189088795E-4</v>
+        <v>6.462035541195477E-4</v>
       </c>
       <c r="G28" t="n" s="0">
-        <v>5.106111377054412E-4</v>
+        <v>5.107986016888279E-4</v>
       </c>
       <c r="H28" t="n" s="0">
-        <v>1.287021991988288E-4</v>
+        <v>2.572678157962439E-4</v>
       </c>
     </row>
     <row r="29">
@@ -908,13 +908,13 @@
         <v>17</v>
       </c>
       <c r="F29" t="n" s="0">
-        <v>0.0011666531637365308</v>
+        <v>5.183613302447638E-4</v>
       </c>
       <c r="G29" t="n" s="0">
-        <v>1.2826062559120131E-4</v>
+        <v>5.129602616097335E-4</v>
       </c>
       <c r="H29" t="n" s="0">
-        <v>0.0</v>
+        <v>1.2715770734653654E-4</v>
       </c>
     </row>
     <row r="30">
@@ -934,13 +934,13 @@
         <v>15</v>
       </c>
       <c r="F30" t="n" s="0">
-        <v>5.077672521857793E-4</v>
+        <v>6.350718425021831E-4</v>
       </c>
       <c r="G30" t="n" s="0">
-        <v>7.577671129072998E-4</v>
+        <v>0.0011354675918624822</v>
       </c>
       <c r="H30" t="n" s="0">
-        <v>3.8441824705279346E-4</v>
+        <v>3.8442440454261503E-4</v>
       </c>
     </row>
     <row r="31">
@@ -960,13 +960,13 @@
         <v>16</v>
       </c>
       <c r="F31" t="n" s="0">
-        <v>1.2871462359017265E-4</v>
+        <v>0.0</v>
       </c>
       <c r="G31" t="n" s="0">
-        <v>0.00102989926297834</v>
+        <v>7.724866021854934E-4</v>
       </c>
       <c r="H31" t="n" s="0">
-        <v>6.395702088196731E-4</v>
+        <v>6.398259673368843E-4</v>
       </c>
     </row>
     <row r="32">
@@ -1142,13 +1142,13 @@
         <v>16</v>
       </c>
       <c r="F38" t="n" s="0">
-        <v>0.005948990570217075</v>
+        <v>0.007347934185313633</v>
       </c>
       <c r="G38" t="n" s="0">
-        <v>0.004096131076194438</v>
+        <v>0.005871840694408987</v>
       </c>
       <c r="H38" t="n" s="0">
-        <v>0.007947316979378635</v>
+        <v>0.008900557085227637</v>
       </c>
     </row>
     <row r="39">
@@ -1168,13 +1168,13 @@
         <v>17</v>
       </c>
       <c r="F39" t="n" s="0">
-        <v>0.007025611547550616</v>
+        <v>0.006650360494300833</v>
       </c>
       <c r="G39" t="n" s="0">
-        <v>0.0035148812913934225</v>
+        <v>0.0031200234001755012</v>
       </c>
       <c r="H39" t="n" s="0">
-        <v>0.005319235197768516</v>
+        <v>0.005585775757083705</v>
       </c>
     </row>
     <row r="40">
@@ -1194,13 +1194,13 @@
         <v>15</v>
       </c>
       <c r="F40" t="n" s="0">
-        <v>0.006976518846290494</v>
+        <v>0.006605255063219414</v>
       </c>
       <c r="G40" t="n" s="0">
-        <v>0.009289895647747518</v>
+        <v>0.010143864238093719</v>
       </c>
       <c r="H40" t="n" s="0">
-        <v>0.003605749883296042</v>
+        <v>0.005269076305220883</v>
       </c>
     </row>
     <row r="41">
@@ -1220,13 +1220,13 @@
         <v>17</v>
       </c>
       <c r="F41" t="n" s="0">
-        <v>0.005329087393783814</v>
+        <v>0.007588286798326686</v>
       </c>
       <c r="G41" t="n" s="0">
-        <v>0.006522781774580336</v>
+        <v>0.004994717126116608</v>
       </c>
       <c r="H41" t="n" s="0">
-        <v>0.004196004259580082</v>
+        <v>0.004198406513891318</v>
       </c>
     </row>
     <row r="42">
@@ -1246,13 +1246,13 @@
         <v>15</v>
       </c>
       <c r="F42" t="n" s="0">
-        <v>0.0064747516424921445</v>
+        <v>0.008999017712855287</v>
       </c>
       <c r="G42" t="n" s="0">
-        <v>0.009526212857232982</v>
+        <v>0.007145341300705049</v>
       </c>
       <c r="H42" t="n" s="0">
-        <v>0.007431371920945578</v>
+        <v>0.00762563880745262</v>
       </c>
     </row>
     <row r="43">
@@ -1272,13 +1272,13 @@
         <v>16</v>
       </c>
       <c r="F43" t="n" s="0">
-        <v>0.004630597314896696</v>
+        <v>0.005135117786764234</v>
       </c>
       <c r="G43" t="n" s="0">
-        <v>0.006258165454281521</v>
+        <v>0.005851431510923208</v>
       </c>
       <c r="H43" t="n" s="0">
-        <v>0.006907026940602766</v>
+        <v>0.007560831050667179</v>
       </c>
     </row>
     <row r="44">
@@ -1454,13 +1454,13 @@
         <v>16</v>
       </c>
       <c r="F50" t="n" s="0">
-        <v>0.034867900648631545</v>
+        <v>0.034617021611993</v>
       </c>
       <c r="G50" t="n" s="0">
-        <v>0.025415881733133243</v>
+        <v>0.028848148325435197</v>
       </c>
       <c r="H50" t="n" s="0">
-        <v>0.03751997443272611</v>
+        <v>0.03644338375205599</v>
       </c>
     </row>
     <row r="51">
@@ -1480,13 +1480,13 @@
         <v>17</v>
       </c>
       <c r="F51" t="n" s="0">
-        <v>0.03267589517013398</v>
+        <v>0.033485298556065635</v>
       </c>
       <c r="G51" t="n" s="0">
-        <v>0.02916356817226551</v>
+        <v>0.02871755158672539</v>
       </c>
       <c r="H51" t="n" s="0">
-        <v>0.030438529454805612</v>
+        <v>0.03264618722977022</v>
       </c>
     </row>
     <row r="52">
@@ -1506,13 +1506,13 @@
         <v>15</v>
       </c>
       <c r="F52" t="n" s="0">
-        <v>0.028972854117152513</v>
+        <v>0.035049146404552506</v>
       </c>
       <c r="G52" t="n" s="0">
-        <v>0.03702226123035187</v>
+        <v>0.0340498929951768</v>
       </c>
       <c r="H52" t="n" s="0">
-        <v>0.02234023663863376</v>
+        <v>0.02643894437207507</v>
       </c>
     </row>
     <row r="53">
@@ -1532,13 +1532,13 @@
         <v>17</v>
       </c>
       <c r="F53" t="n" s="0">
-        <v>0.030806726785279064</v>
+        <v>0.0302985876948639</v>
       </c>
       <c r="G53" t="n" s="0">
-        <v>0.03664879825663703</v>
+        <v>0.03818432264471282</v>
       </c>
       <c r="H53" t="n" s="0">
-        <v>0.028999423852506243</v>
+        <v>0.028090066562629384</v>
       </c>
     </row>
     <row r="54">
@@ -1558,13 +1558,13 @@
         <v>15</v>
       </c>
       <c r="F54" t="n" s="0">
-        <v>0.030295812890010956</v>
+        <v>0.03593762368400222</v>
       </c>
       <c r="G54" t="n" s="0">
-        <v>0.038636651068673325</v>
+        <v>0.03853442830069488</v>
       </c>
       <c r="H54" t="n" s="0">
-        <v>0.03583182161146875</v>
+        <v>0.037966795033636404</v>
       </c>
     </row>
     <row r="55">
@@ -1584,13 +1584,13 @@
         <v>16</v>
       </c>
       <c r="F55" t="n" s="0">
-        <v>0.02809240417226595</v>
+        <v>0.0307120187221492</v>
       </c>
       <c r="G55" t="n" s="0">
-        <v>0.03130384373842611</v>
+        <v>0.03288216688341923</v>
       </c>
       <c r="H55" t="n" s="0">
-        <v>0.03610499792683316</v>
+        <v>0.035239180319976894</v>
       </c>
     </row>
     <row r="56">
@@ -1636,13 +1636,13 @@
         <v>10</v>
       </c>
       <c r="F57" t="n" s="0">
-        <v>4.271986714121319E-4</v>
+        <v>4.0587558311237147E-4</v>
       </c>
       <c r="G57" t="n" s="0">
-        <v>4.480107522580542E-4</v>
+        <v>5.333120008532992E-4</v>
       </c>
       <c r="H57" t="n" s="0">
-        <v>2.1376599570864762E-4</v>
+        <v>3.6349252167591436E-4</v>
       </c>
     </row>
     <row r="58">
@@ -1688,13 +1688,13 @@
         <v>10</v>
       </c>
       <c r="F59" t="n" s="0">
-        <v>0.006066561285085658</v>
+        <v>0.0070586287999530135</v>
       </c>
       <c r="G59" t="n" s="0">
-        <v>0.0065533876958545016</v>
+        <v>0.006199995197938315</v>
       </c>
       <c r="H59" t="n" s="0">
-        <v>0.005902212527766863</v>
+        <v>0.006523506010180947</v>
       </c>
     </row>
     <row r="60">
@@ -1740,13 +1740,13 @@
         <v>10</v>
       </c>
       <c r="F61" t="n" s="0">
-        <v>0.030964177337379405</v>
+        <v>0.0333647844002708</v>
       </c>
       <c r="G61" t="n" s="0">
-        <v>0.03305406449378638</v>
+        <v>0.033551199418076404</v>
       </c>
       <c r="H61" t="n" s="0">
-        <v>0.03189179493083239</v>
+        <v>0.032801276080975474</v>
       </c>
     </row>
   </sheetData>
@@ -1828,13 +1828,13 @@
         <v>21</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>0.33856359889911514</v>
+        <v>0.33852137203940996</v>
       </c>
       <c r="F3" t="n" s="0">
-        <v>0.33669268777550493</v>
+        <v>0.33655202994594186</v>
       </c>
       <c r="G3" t="n" s="0">
-        <v>0.3360517502643841</v>
+        <v>0.3359996130903889</v>
       </c>
     </row>
     <row r="4">
@@ -1874,13 +1874,13 @@
         <v>21</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>0.43759398252210135</v>
+        <v>0.4376993531710139</v>
       </c>
       <c r="F5" t="n" s="0">
-        <v>0.4350355800575587</v>
+        <v>0.435272997551947</v>
       </c>
       <c r="G5" t="n" s="0">
-        <v>0.43541319106554505</v>
+        <v>0.43490065608219797</v>
       </c>
     </row>
     <row r="6">
@@ -1920,13 +1920,13 @@
         <v>21</v>
       </c>
       <c r="E7" t="n" s="0">
-        <v>0.5269323635404631</v>
+        <v>0.5264678502525039</v>
       </c>
       <c r="F7" t="n" s="0">
-        <v>0.5242546703555414</v>
+        <v>0.5243055200960531</v>
       </c>
       <c r="G7" t="n" s="0">
-        <v>0.5229660698177806</v>
+        <v>0.5222178891542923</v>
       </c>
     </row>
     <row r="8">
@@ -1966,13 +1966,13 @@
         <v>23</v>
       </c>
       <c r="E9" t="n" s="0">
-        <v>0.33856359889910764</v>
+        <v>0.33852137203939875</v>
       </c>
       <c r="F9" t="n" s="0">
-        <v>0.3366926877754882</v>
+        <v>0.3365520299459195</v>
       </c>
       <c r="G9" t="n" s="0">
-        <v>0.33605175026438505</v>
+        <v>0.3359996130903881</v>
       </c>
     </row>
     <row r="10">
@@ -2012,13 +2012,13 @@
         <v>23</v>
       </c>
       <c r="E11" t="n" s="0">
-        <v>0.4375939825221054</v>
+        <v>0.43769935317101477</v>
       </c>
       <c r="F11" t="n" s="0">
-        <v>0.43503558005755605</v>
+        <v>0.43527299755195853</v>
       </c>
       <c r="G11" t="n" s="0">
-        <v>0.4354131910655258</v>
+        <v>0.4349006560821824</v>
       </c>
     </row>
     <row r="12">
@@ -2058,13 +2058,13 @@
         <v>23</v>
       </c>
       <c r="E13" t="n" s="0">
-        <v>0.5269323635404545</v>
+        <v>0.5264678502525227</v>
       </c>
       <c r="F13" t="n" s="0">
-        <v>0.5242546703555285</v>
+        <v>0.5243055200960446</v>
       </c>
       <c r="G13" t="n" s="0">
-        <v>0.5229660698177991</v>
+        <v>0.5222178891542767</v>
       </c>
     </row>
     <row r="14">
@@ -2219,13 +2219,13 @@
         <v>25</v>
       </c>
       <c r="E20" t="n" s="0">
-        <v>0.3320179811105222</v>
+        <v>0.33147462931310007</v>
       </c>
       <c r="F20" t="n" s="0">
-        <v>0.3347973600400259</v>
+        <v>0.3345128185250108</v>
       </c>
       <c r="G20" t="n" s="0">
-        <v>0.33165532185139296</v>
+        <v>0.33188024049731923</v>
       </c>
     </row>
     <row r="21">
@@ -2242,13 +2242,13 @@
         <v>26</v>
       </c>
       <c r="E21" t="n" s="0">
-        <v>0.3413114744390392</v>
+        <v>0.3411748187829399</v>
       </c>
       <c r="F21" t="n" s="0">
-        <v>0.34132405347741784</v>
+        <v>0.341404088337719</v>
       </c>
       <c r="G21" t="n" s="0">
-        <v>0.33958105487771</v>
+        <v>0.3394117055305211</v>
       </c>
     </row>
     <row r="22">
@@ -2265,13 +2265,13 @@
         <v>27</v>
       </c>
       <c r="E22" t="n" s="0">
-        <v>0.3479959907926321</v>
+        <v>0.34779077080152854</v>
       </c>
       <c r="F22" t="n" s="0">
-        <v>0.33669556006716267</v>
+        <v>0.3367314084480059</v>
       </c>
       <c r="G22" t="n" s="0">
-        <v>0.34022730801218165</v>
+        <v>0.3401338206546221</v>
       </c>
     </row>
     <row r="23">
@@ -2288,13 +2288,13 @@
         <v>28</v>
       </c>
       <c r="E23" t="n" s="0">
-        <v>0.33489673451086216</v>
+        <v>0.3351056375614422</v>
       </c>
       <c r="F23" t="n" s="0">
-        <v>0.3348052400103547</v>
+        <v>0.3352159455830176</v>
       </c>
       <c r="G23" t="n" s="0">
-        <v>0.3365553226782217</v>
+        <v>0.33664115452024834</v>
       </c>
     </row>
     <row r="24">
@@ -2311,13 +2311,13 @@
         <v>29</v>
       </c>
       <c r="E24" t="n" s="0">
-        <v>0.3382090468736608</v>
+        <v>0.33832746410736414</v>
       </c>
       <c r="F24" t="n" s="0">
-        <v>0.3335706002148202</v>
+        <v>0.33306029314778185</v>
       </c>
       <c r="G24" t="n" s="0">
-        <v>0.33457886035452694</v>
+        <v>0.3344834591849551</v>
       </c>
     </row>
     <row r="25">
@@ -2334,13 +2334,13 @@
         <v>30</v>
       </c>
       <c r="E25" t="n" s="0">
-        <v>0.33695036566790876</v>
+        <v>0.3372549116700212</v>
       </c>
       <c r="F25" t="n" s="0">
-        <v>0.33896331284321063</v>
+        <v>0.33838762563406694</v>
       </c>
       <c r="G25" t="n" s="0">
-        <v>0.333712633812275</v>
+        <v>0.33344729815464325</v>
       </c>
     </row>
     <row r="26">
@@ -2495,13 +2495,13 @@
         <v>25</v>
       </c>
       <c r="E32" t="n" s="0">
-        <v>0.4286348279298464</v>
+        <v>0.4275965760380635</v>
       </c>
       <c r="F32" t="n" s="0">
-        <v>0.43372297409253185</v>
+        <v>0.43241917823131093</v>
       </c>
       <c r="G32" t="n" s="0">
-        <v>0.42939487545393423</v>
+        <v>0.43066415707025313</v>
       </c>
     </row>
     <row r="33">
@@ -2518,13 +2518,13 @@
         <v>26</v>
       </c>
       <c r="E33" t="n" s="0">
-        <v>0.4416764864988256</v>
+        <v>0.4416138126156112</v>
       </c>
       <c r="F33" t="n" s="0">
-        <v>0.4401373520817956</v>
+        <v>0.44105201186134335</v>
       </c>
       <c r="G33" t="n" s="0">
-        <v>0.4397102318455569</v>
+        <v>0.4381168995854479</v>
       </c>
     </row>
     <row r="34">
@@ -2541,13 +2541,13 @@
         <v>27</v>
       </c>
       <c r="E34" t="n" s="0">
-        <v>0.44900950914482074</v>
+        <v>0.4489931769667431</v>
       </c>
       <c r="F34" t="n" s="0">
-        <v>0.4358336138416358</v>
+        <v>0.43516117202235394</v>
       </c>
       <c r="G34" t="n" s="0">
-        <v>0.4392691290713604</v>
+        <v>0.43913769604546626</v>
       </c>
     </row>
     <row r="35">
@@ -2564,13 +2564,13 @@
         <v>28</v>
       </c>
       <c r="E35" t="n" s="0">
-        <v>0.4340999655272012</v>
+        <v>0.43443074111764257</v>
       </c>
       <c r="F35" t="n" s="0">
-        <v>0.43152417153089606</v>
+        <v>0.4339797778045631</v>
       </c>
       <c r="G35" t="n" s="0">
-        <v>0.43698315640767577</v>
+        <v>0.43558236111626725</v>
       </c>
     </row>
     <row r="36">
@@ -2587,13 +2587,13 @@
         <v>29</v>
       </c>
       <c r="E36" t="n" s="0">
-        <v>0.43688903226142084</v>
+        <v>0.4369394540677475</v>
       </c>
       <c r="F36" t="n" s="0">
-        <v>0.4296125548106518</v>
+        <v>0.4295324982265844</v>
       </c>
       <c r="G36" t="n" s="0">
-        <v>0.4334062738965905</v>
+        <v>0.4315669863401897</v>
       </c>
     </row>
     <row r="37">
@@ -2610,13 +2610,13 @@
         <v>30</v>
       </c>
       <c r="E37" t="n" s="0">
-        <v>0.4352540737705597</v>
+        <v>0.4366223582202841</v>
       </c>
       <c r="F37" t="n" s="0">
-        <v>0.43938281398782814</v>
+        <v>0.43949334716552096</v>
       </c>
       <c r="G37" t="n" s="0">
-        <v>0.43371547971814917</v>
+        <v>0.4343358363355529</v>
       </c>
     </row>
     <row r="38">
@@ -2771,13 +2771,13 @@
         <v>25</v>
       </c>
       <c r="E44" t="n" s="0">
-        <v>0.513487038536892</v>
+        <v>0.5142180114597392</v>
       </c>
       <c r="F44" t="n" s="0">
-        <v>0.5214350057827569</v>
+        <v>0.5187264775129068</v>
       </c>
       <c r="G44" t="n" s="0">
-        <v>0.5171634628025559</v>
+        <v>0.5184380821323742</v>
       </c>
     </row>
     <row r="45">
@@ -2794,13 +2794,13 @@
         <v>26</v>
       </c>
       <c r="E45" t="n" s="0">
-        <v>0.5313908036384258</v>
+        <v>0.5317968072607728</v>
       </c>
       <c r="F45" t="n" s="0">
-        <v>0.529157311816764</v>
+        <v>0.5318513881084865</v>
       </c>
       <c r="G45" t="n" s="0">
-        <v>0.525567550097013</v>
+        <v>0.5244101894702281</v>
       </c>
     </row>
     <row r="46">
@@ -2817,13 +2817,13 @@
         <v>27</v>
       </c>
       <c r="E46" t="n" s="0">
-        <v>0.5389521763247812</v>
+        <v>0.5407102337400326</v>
       </c>
       <c r="F46" t="n" s="0">
-        <v>0.523539197492089</v>
+        <v>0.5256264907520948</v>
       </c>
       <c r="G46" t="n" s="0">
-        <v>0.52947961961584</v>
+        <v>0.523405521252446</v>
       </c>
     </row>
     <row r="47">
@@ -2840,13 +2840,13 @@
         <v>28</v>
       </c>
       <c r="E47" t="n" s="0">
-        <v>0.5248519155729368</v>
+        <v>0.5230895497983737</v>
       </c>
       <c r="F47" t="n" s="0">
-        <v>0.521860647786502</v>
+        <v>0.5234828687890548</v>
       </c>
       <c r="G47" t="n" s="0">
-        <v>0.5255246579748025</v>
+        <v>0.5225017849994579</v>
       </c>
     </row>
     <row r="48">
@@ -2863,13 +2863,13 @@
         <v>29</v>
       </c>
       <c r="E48" t="n" s="0">
-        <v>0.5291668704857422</v>
+        <v>0.5286889694379902</v>
       </c>
       <c r="F48" t="n" s="0">
-        <v>0.5195314161867935</v>
+        <v>0.5219163568771427</v>
       </c>
       <c r="G48" t="n" s="0">
-        <v>0.5205958393031536</v>
+        <v>0.5222242326252909</v>
       </c>
     </row>
     <row r="49">
@@ -2886,13 +2886,13 @@
         <v>30</v>
       </c>
       <c r="E49" t="n" s="0">
-        <v>0.523745376683999</v>
+        <v>0.5203035298181679</v>
       </c>
       <c r="F49" t="n" s="0">
-        <v>0.5300044430683872</v>
+        <v>0.5242295385367275</v>
       </c>
       <c r="G49" t="n" s="0">
-        <v>0.5194652891132777</v>
+        <v>0.5223275244459676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>